<commit_message>
fix spelling error in excel file: efficencyDropPerYear to efficiencyDropPerYear
</commit_message>
<xml_diff>
--- a/reskit/csp/data/CSP_database.xlsx
+++ b/reskit/csp/data/CSP_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DCE6A~1.FRA\DOCUME~1\MobaXterm\slash\RemoteFiles\67580_2_145\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\ethos_reskit_wind_validation_2025\env\RESKit\reskit\csp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF8C1A2-6BBC-472D-B5DA-7743EB1B887E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3250A6E-4EB0-45FD-954A-55B423B62BFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16920" xr2:uid="{EF8FF396-6CE6-4D67-BA8C-A21BECB15794}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{EF8FF396-6CE6-4D67-BA8C-A21BECB15794}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -322,9 +322,6 @@
     <t>Validation_9</t>
   </si>
   <si>
-    <t>efficencyDropPerYear</t>
-  </si>
-  <si>
     <t>lifetime</t>
   </si>
   <si>
@@ -506,6 +503,9 @@
   </si>
   <si>
     <t>Dataset_Heliosol_2030_validation3</t>
+  </si>
+  <si>
+    <t>efficiencyDropPerYear</t>
   </si>
 </sst>
 </file>
@@ -604,27 +604,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -643,9 +638,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -683,7 +678,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -789,7 +784,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -931,7 +926,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -998,58 +993,58 @@
         <v>75</v>
       </c>
       <c r="N1" t="s">
+        <v>80</v>
+      </c>
+      <c r="O1" t="s">
+        <v>79</v>
+      </c>
+      <c r="P1" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q1" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="R1" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="S1" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="T1" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="U1" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="V1" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="W1" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="X1" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="Y1" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="Z1" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="AA1" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="AB1" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="AC1" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AD1" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="AE1" t="s">
         <v>81</v>
-      </c>
-      <c r="O1" t="s">
-        <v>80</v>
-      </c>
-      <c r="P1" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q1" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="R1" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="S1" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="T1" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="U1" s="14" t="s">
-        <v>116</v>
-      </c>
-      <c r="V1" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="W1" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="X1" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="Y1" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="Z1" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="AA1" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="AB1" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="AC1" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="AD1" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:31">
@@ -1093,52 +1088,52 @@
         <v>75</v>
       </c>
       <c r="N2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O2" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q2" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="R2" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="S2" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="T2" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="U2" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="V2" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="W2" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="X2" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="Y2" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="Z2" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="AA2" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="AB2" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="AC2" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="AD2" s="15" t="s">
-        <v>101</v>
+        <v>79</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="R2" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="S2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="T2" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="U2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="V2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="W2" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="X2" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="Z2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="AA2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="AB2" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="AC2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="AD2" s="11" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:31">
@@ -1154,7 +1149,7 @@
       <c r="D3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="4" t="s">
         <v>40</v>
       </c>
       <c r="F3" t="s">
@@ -1190,50 +1185,50 @@
       <c r="P3" t="s">
         <v>18</v>
       </c>
-      <c r="Q3" s="13" t="s">
+      <c r="Q3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="R3" s="13" t="s">
+      <c r="R3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="S3" s="13" t="s">
+      <c r="S3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="T3" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="U3" s="13" t="s">
+      <c r="T3" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="U3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="V3" s="13" t="s">
+      <c r="V3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="W3" s="13" t="s">
+      <c r="W3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="X3" s="13" t="s">
+      <c r="X3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="Y3" s="13" t="s">
+      <c r="Y3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="Z3" s="13" t="s">
+      <c r="Z3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="AA3" s="13" t="s">
+      <c r="AA3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="AB3" s="13" t="s">
+      <c r="AB3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="AC3" s="13" t="s">
+      <c r="AC3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="AD3" s="13" t="s">
+      <c r="AD3" s="9" t="s">
         <v>18</v>
       </c>
       <c r="AE3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:31">
@@ -1249,7 +1244,7 @@
       <c r="D4">
         <v>8.8400000000000002E-4</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="5">
         <v>8.4924000000000002E-5</v>
       </c>
       <c r="F4" s="1">
@@ -1285,50 +1280,50 @@
       <c r="P4" s="1">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="Q4" s="16">
+      <c r="Q4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="R4" s="16">
+      <c r="R4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="S4" s="16">
+      <c r="S4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="T4" s="16">
+      <c r="T4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="U4" s="16">
+      <c r="U4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="V4" s="16">
+      <c r="V4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="W4" s="16">
+      <c r="W4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="X4" s="16">
+      <c r="X4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="Y4" s="16">
+      <c r="Y4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="Z4" s="16">
+      <c r="Z4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="AA4" s="16">
+      <c r="AA4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="AB4" s="16">
+      <c r="AB4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="AC4" s="16">
+      <c r="AC4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
-      <c r="AD4" s="16">
+      <c r="AD4" s="12">
         <v>8.7266462599716496E-5</v>
       </c>
       <c r="AE4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:31">
@@ -1344,7 +1339,7 @@
       <c r="D5">
         <v>5.3690000000000003E-5</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="5">
         <v>3.1093000000000002E-5</v>
       </c>
       <c r="F5" s="1">
@@ -1380,50 +1375,50 @@
       <c r="P5" s="1">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="Q5" s="16">
+      <c r="Q5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="R5" s="16">
+      <c r="R5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="S5" s="16">
+      <c r="S5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="T5" s="16">
+      <c r="T5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="U5" s="16">
+      <c r="U5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="V5" s="16">
+      <c r="V5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="W5" s="16">
+      <c r="W5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="X5" s="16">
+      <c r="X5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="Y5" s="16">
+      <c r="Y5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="Z5" s="16">
+      <c r="Z5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="AA5" s="16">
+      <c r="AA5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="AB5" s="16">
+      <c r="AB5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="AC5" s="16">
+      <c r="AC5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
-      <c r="AD5" s="16">
+      <c r="AD5" s="12">
         <v>3.1070976818244299E-5</v>
       </c>
       <c r="AE5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:31">
@@ -1439,7 +1434,7 @@
       <c r="D6">
         <v>0</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="4">
         <v>0</v>
       </c>
       <c r="F6">
@@ -1475,50 +1470,50 @@
       <c r="P6">
         <v>0</v>
       </c>
-      <c r="Q6" s="15">
-        <v>0</v>
-      </c>
-      <c r="R6" s="15">
-        <v>0</v>
-      </c>
-      <c r="S6" s="15">
-        <v>0</v>
-      </c>
-      <c r="T6" s="15">
-        <v>0</v>
-      </c>
-      <c r="U6" s="15">
-        <v>0</v>
-      </c>
-      <c r="V6" s="15">
-        <v>0</v>
-      </c>
-      <c r="W6" s="15">
-        <v>0</v>
-      </c>
-      <c r="X6" s="15">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="15">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="15">
-        <v>0</v>
-      </c>
-      <c r="AA6" s="15">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="15">
-        <v>0</v>
-      </c>
-      <c r="AC6" s="15">
-        <v>0</v>
-      </c>
-      <c r="AD6" s="15">
+      <c r="Q6" s="11">
+        <v>0</v>
+      </c>
+      <c r="R6" s="11">
+        <v>0</v>
+      </c>
+      <c r="S6" s="11">
+        <v>0</v>
+      </c>
+      <c r="T6" s="11">
+        <v>0</v>
+      </c>
+      <c r="U6" s="11">
+        <v>0</v>
+      </c>
+      <c r="V6" s="11">
+        <v>0</v>
+      </c>
+      <c r="W6" s="11">
+        <v>0</v>
+      </c>
+      <c r="X6" s="11">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="11">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="11">
         <v>0</v>
       </c>
       <c r="AE6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:31">
@@ -1534,7 +1529,7 @@
       <c r="D7">
         <v>0.74199999999999999</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="4">
         <v>0.82699999999999996</v>
       </c>
       <c r="F7">
@@ -1570,50 +1565,50 @@
       <c r="P7">
         <v>0.82699999999999996</v>
       </c>
-      <c r="Q7" s="13">
+      <c r="Q7" s="9">
         <v>0.92688000000000004</v>
       </c>
-      <c r="R7" s="13">
+      <c r="R7" s="9">
         <v>0.92688000000000004</v>
       </c>
-      <c r="S7" s="13">
+      <c r="S7" s="9">
         <v>0.92688000000000004</v>
       </c>
-      <c r="T7" s="13">
+      <c r="T7" s="9">
         <v>0.92688000000000004</v>
       </c>
-      <c r="U7" s="15">
+      <c r="U7" s="11">
         <v>0.82699999999999996</v>
       </c>
-      <c r="V7" s="15">
+      <c r="V7" s="11">
         <v>0.82699999999999996</v>
       </c>
-      <c r="W7" s="13">
+      <c r="W7" s="9">
         <v>0.92688000000000004</v>
       </c>
-      <c r="X7" s="15">
+      <c r="X7" s="11">
         <v>0.82699999999999996</v>
       </c>
-      <c r="Y7" s="15">
+      <c r="Y7" s="11">
         <v>0.82699999999999996</v>
       </c>
-      <c r="Z7" s="15">
+      <c r="Z7" s="11">
         <v>0.82699999999999996</v>
       </c>
-      <c r="AA7" s="15">
+      <c r="AA7" s="11">
         <v>0.82699999999999996</v>
       </c>
-      <c r="AB7" s="15">
+      <c r="AB7" s="11">
         <v>0.82699999999999996</v>
       </c>
-      <c r="AC7" s="15">
+      <c r="AC7" s="11">
         <v>0.82699999999999996</v>
       </c>
-      <c r="AD7" s="15">
+      <c r="AD7" s="11">
         <v>0.82699999999999996</v>
       </c>
       <c r="AE7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:31">
@@ -1629,53 +1624,53 @@
       <c r="D8">
         <v>0.06</v>
       </c>
-      <c r="E8" s="7"/>
+      <c r="E8" s="4"/>
       <c r="O8">
         <v>-1</v>
       </c>
       <c r="P8">
         <v>-1</v>
       </c>
-      <c r="Q8" s="15">
+      <c r="Q8" s="11">
         <v>-1</v>
       </c>
-      <c r="R8" s="15">
+      <c r="R8" s="11">
         <v>-1</v>
       </c>
-      <c r="S8" s="15">
+      <c r="S8" s="11">
         <v>-1</v>
       </c>
-      <c r="T8" s="15">
+      <c r="T8" s="11">
         <v>-1</v>
       </c>
-      <c r="U8" s="15">
+      <c r="U8" s="11">
         <v>-1</v>
       </c>
-      <c r="V8" s="15">
+      <c r="V8" s="11">
         <v>-1</v>
       </c>
-      <c r="W8" s="15">
+      <c r="W8" s="11">
         <v>-1</v>
       </c>
-      <c r="X8" s="15">
+      <c r="X8" s="11">
         <v>-1</v>
       </c>
-      <c r="Y8" s="15">
+      <c r="Y8" s="11">
         <v>-1</v>
       </c>
-      <c r="Z8" s="15">
+      <c r="Z8" s="11">
         <v>-1</v>
       </c>
-      <c r="AA8" s="15">
+      <c r="AA8" s="11">
         <v>-1</v>
       </c>
-      <c r="AB8" s="15">
+      <c r="AB8" s="11">
         <v>-1</v>
       </c>
-      <c r="AC8" s="15">
+      <c r="AC8" s="11">
         <v>-1</v>
       </c>
-      <c r="AD8" s="15">
+      <c r="AD8" s="11">
         <v>-1</v>
       </c>
     </row>
@@ -1728,50 +1723,50 @@
       <c r="P9">
         <v>16</v>
       </c>
-      <c r="Q9" s="15">
+      <c r="Q9" s="11">
         <v>16</v>
       </c>
-      <c r="R9" s="15">
+      <c r="R9" s="11">
         <v>16</v>
       </c>
-      <c r="S9" s="15">
+      <c r="S9" s="11">
         <v>16</v>
       </c>
-      <c r="T9" s="15">
+      <c r="T9" s="11">
         <v>16</v>
       </c>
-      <c r="U9" s="15">
+      <c r="U9" s="11">
         <v>16</v>
       </c>
-      <c r="V9" s="15">
+      <c r="V9" s="11">
         <v>16</v>
       </c>
-      <c r="W9" s="15">
+      <c r="W9" s="11">
         <v>16</v>
       </c>
-      <c r="X9" s="15">
+      <c r="X9" s="11">
         <v>16</v>
       </c>
-      <c r="Y9" s="15">
+      <c r="Y9" s="11">
         <v>16</v>
       </c>
-      <c r="Z9" s="15">
+      <c r="Z9" s="11">
         <v>16</v>
       </c>
-      <c r="AA9" s="15">
+      <c r="AA9" s="11">
         <v>16</v>
       </c>
-      <c r="AB9" s="15">
+      <c r="AB9" s="11">
         <v>16</v>
       </c>
-      <c r="AC9" s="15">
+      <c r="AC9" s="11">
         <v>16</v>
       </c>
-      <c r="AD9" s="15">
+      <c r="AD9" s="11">
         <v>16</v>
       </c>
       <c r="AE9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:31">
@@ -1823,50 +1818,50 @@
       <c r="P10">
         <v>0</v>
       </c>
-      <c r="Q10" s="15">
-        <v>0</v>
-      </c>
-      <c r="R10" s="15">
-        <v>0</v>
-      </c>
-      <c r="S10" s="15">
-        <v>0</v>
-      </c>
-      <c r="T10" s="15">
-        <v>0</v>
-      </c>
-      <c r="U10" s="15">
-        <v>0</v>
-      </c>
-      <c r="V10" s="15">
-        <v>0</v>
-      </c>
-      <c r="W10" s="15">
-        <v>0</v>
-      </c>
-      <c r="X10" s="15">
-        <v>0</v>
-      </c>
-      <c r="Y10" s="15">
-        <v>0</v>
-      </c>
-      <c r="Z10" s="15">
-        <v>0</v>
-      </c>
-      <c r="AA10" s="15">
-        <v>0</v>
-      </c>
-      <c r="AB10" s="15">
-        <v>0</v>
-      </c>
-      <c r="AC10" s="15">
-        <v>0</v>
-      </c>
-      <c r="AD10" s="15">
+      <c r="Q10" s="11">
+        <v>0</v>
+      </c>
+      <c r="R10" s="11">
+        <v>0</v>
+      </c>
+      <c r="S10" s="11">
+        <v>0</v>
+      </c>
+      <c r="T10" s="11">
+        <v>0</v>
+      </c>
+      <c r="U10" s="11">
+        <v>0</v>
+      </c>
+      <c r="V10" s="11">
+        <v>0</v>
+      </c>
+      <c r="W10" s="11">
+        <v>0</v>
+      </c>
+      <c r="X10" s="11">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="11">
+        <v>0</v>
+      </c>
+      <c r="AD10" s="11">
         <v>0</v>
       </c>
       <c r="AE10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:31">
@@ -1918,50 +1913,50 @@
       <c r="P11">
         <v>4.4701935910452829E-2</v>
       </c>
-      <c r="Q11" s="15">
+      <c r="Q11" s="11">
         <v>4.4701935910452829E-2</v>
       </c>
-      <c r="R11" s="15">
+      <c r="R11" s="11">
         <v>4.4701935910452802E-2</v>
       </c>
-      <c r="S11" s="15">
+      <c r="S11" s="11">
         <v>4.4701935910452829E-2</v>
       </c>
-      <c r="T11" s="15">
+      <c r="T11" s="11">
         <v>4.4701935910452802E-2</v>
       </c>
-      <c r="U11" s="15">
+      <c r="U11" s="11">
         <v>4.4701935910452829E-2</v>
       </c>
-      <c r="V11" s="15">
+      <c r="V11" s="11">
         <v>4.4701935910452829E-2</v>
       </c>
-      <c r="W11" s="15">
+      <c r="W11" s="11">
         <v>4.4701935910452802E-2</v>
       </c>
-      <c r="X11" s="15">
+      <c r="X11" s="11">
         <v>4.4701935910452802E-2</v>
       </c>
-      <c r="Y11" s="15">
+      <c r="Y11" s="11">
         <v>4.4701935910452829E-2</v>
       </c>
-      <c r="Z11" s="15">
+      <c r="Z11" s="11">
         <v>4.4701935910452829E-2</v>
       </c>
-      <c r="AA11" s="15">
+      <c r="AA11" s="11">
         <v>4.4701935910452829E-2</v>
       </c>
-      <c r="AB11" s="15">
+      <c r="AB11" s="11">
         <v>4.4701935910452802E-2</v>
       </c>
-      <c r="AC11" s="15">
+      <c r="AC11" s="11">
         <v>4.4701935910452829E-2</v>
       </c>
-      <c r="AD11" s="15">
+      <c r="AD11" s="11">
         <v>4.4701935910452802E-2</v>
       </c>
       <c r="AE11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:31">
@@ -2013,50 +2008,50 @@
       <c r="P12">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="Q12" s="15">
+      <c r="Q12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="R12" s="15">
+      <c r="R12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="S12" s="15">
+      <c r="S12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="T12" s="15">
+      <c r="T12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="U12" s="15">
+      <c r="U12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="V12" s="15">
+      <c r="V12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="W12" s="15">
+      <c r="W12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="X12" s="15">
+      <c r="X12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="Y12" s="15">
+      <c r="Y12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="Z12" s="15">
+      <c r="Z12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="AA12" s="15">
+      <c r="AA12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="AB12" s="15">
+      <c r="AB12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="AC12" s="15">
+      <c r="AC12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
-      <c r="AD12" s="15">
+      <c r="AD12" s="11">
         <v>-2.9278818932777496E-4</v>
       </c>
       <c r="AE12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:31">
@@ -2108,50 +2103,50 @@
       <c r="P13">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="Q13" s="15">
+      <c r="Q13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="R13" s="15">
+      <c r="R13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="S13" s="15">
+      <c r="S13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="T13" s="15">
+      <c r="T13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="U13" s="15">
+      <c r="U13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="V13" s="15">
+      <c r="V13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="W13" s="15">
+      <c r="W13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="X13" s="15">
+      <c r="X13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="Y13" s="15">
+      <c r="Y13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="Z13" s="15">
+      <c r="Z13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="AA13" s="15">
+      <c r="AA13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="AB13" s="15">
+      <c r="AB13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="AC13" s="15">
+      <c r="AC13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
-      <c r="AD13" s="15">
+      <c r="AD13" s="11">
         <v>1.2085236947426394E-6</v>
       </c>
       <c r="AE13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" spans="1:31">
@@ -2203,50 +2198,50 @@
       <c r="P14">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="Q14" s="15">
+      <c r="Q14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="R14" s="15">
+      <c r="R14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="S14" s="15">
+      <c r="S14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="T14" s="15">
+      <c r="T14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="U14" s="15">
+      <c r="U14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="V14" s="15">
+      <c r="V14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="W14" s="15">
+      <c r="W14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="X14" s="15">
+      <c r="X14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="Y14" s="15">
+      <c r="Y14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="Z14" s="15">
+      <c r="Z14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="AA14" s="15">
+      <c r="AA14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="AB14" s="15">
+      <c r="AB14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="AC14" s="15">
+      <c r="AC14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
-      <c r="AD14" s="15">
+      <c r="AD14" s="11">
         <v>-4.6531969642924003E-10</v>
       </c>
       <c r="AE14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:31">
@@ -2262,7 +2257,7 @@
       <c r="D15">
         <v>909060</v>
       </c>
-      <c r="E15" s="7">
+      <c r="E15" s="4">
         <v>1372800</v>
       </c>
       <c r="F15">
@@ -2292,56 +2287,56 @@
       <c r="N15">
         <v>1372800</v>
       </c>
-      <c r="O15" s="13"/>
-      <c r="P15" s="9">
+      <c r="O15" s="9"/>
+      <c r="P15">
         <v>1200000</v>
       </c>
-      <c r="Q15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="R15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="S15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="T15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="U15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="V15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="W15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="X15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="Y15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="Z15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="AA15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="AB15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="AC15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="AD15" s="15" t="s">
-        <v>99</v>
+      <c r="Q15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="R15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="S15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="T15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="U15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="V15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="W15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="X15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="Y15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="Z15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="AB15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="AC15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="AD15" s="11" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:31">
       <c r="A16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B16" s="3">
         <v>1</v>
@@ -2349,89 +2344,89 @@
       <c r="C16" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="6">
         <v>0.38300000000000001</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="7">
         <v>0.30509999999999998</v>
       </c>
-      <c r="F16" s="10">
+      <c r="F16" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="G16" s="10">
+      <c r="G16" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="H16" s="10">
+      <c r="H16" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="I16" s="10">
+      <c r="I16" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="J16" s="10">
+      <c r="J16" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="K16" s="10">
+      <c r="K16" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="L16" s="10">
+      <c r="L16" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="M16" s="10">
+      <c r="M16" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="N16" s="11">
+      <c r="N16" s="7">
         <v>0.434</v>
       </c>
-      <c r="O16" s="13"/>
-      <c r="P16" s="9">
+      <c r="O16" s="9"/>
+      <c r="P16">
         <v>0.38300000000000001</v>
       </c>
-      <c r="Q16" s="15">
+      <c r="Q16" s="11">
         <v>0.38</v>
       </c>
-      <c r="R16" s="15">
+      <c r="R16" s="11">
         <v>0.38</v>
       </c>
-      <c r="S16" s="15">
+      <c r="S16" s="11">
         <v>0.38</v>
       </c>
-      <c r="T16" s="15">
+      <c r="T16" s="11">
         <v>0.38</v>
       </c>
-      <c r="U16" s="15">
+      <c r="U16" s="11">
         <v>0.38</v>
       </c>
-      <c r="V16" s="15">
+      <c r="V16" s="11">
         <v>0.38</v>
       </c>
-      <c r="W16" s="15">
+      <c r="W16" s="11">
         <v>0.38</v>
       </c>
-      <c r="X16" s="15">
+      <c r="X16" s="11">
         <v>0.38</v>
       </c>
-      <c r="Y16" s="15">
+      <c r="Y16" s="11">
         <v>0.38</v>
       </c>
-      <c r="Z16" s="15">
+      <c r="Z16" s="11">
         <v>0.38</v>
       </c>
-      <c r="AA16" s="15">
+      <c r="AA16" s="11">
         <v>0.38</v>
       </c>
-      <c r="AB16" s="15">
+      <c r="AB16" s="11">
         <v>0.38</v>
       </c>
-      <c r="AC16" s="15">
+      <c r="AC16" s="11">
         <v>0.38</v>
       </c>
-      <c r="AD16" s="15">
+      <c r="AD16" s="11">
         <v>0.38</v>
       </c>
     </row>
     <row r="17" spans="1:31">
       <c r="A17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B17" s="3">
         <v>1</v>
@@ -2439,83 +2434,83 @@
       <c r="C17" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="6">
         <v>0.38300000000000001</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="7">
         <v>0.30509999999999998</v>
       </c>
-      <c r="F17" s="10">
+      <c r="F17" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="G17" s="10">
+      <c r="G17" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="H17" s="10">
+      <c r="H17" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="I17" s="10">
+      <c r="I17" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="J17" s="10">
+      <c r="J17" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="K17" s="10">
+      <c r="K17" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="L17" s="10">
+      <c r="L17" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="M17" s="10">
+      <c r="M17" s="6">
         <v>0.30509999999999998</v>
       </c>
-      <c r="N17" s="11">
+      <c r="N17" s="7">
         <v>0.434</v>
       </c>
-      <c r="O17" s="13"/>
-      <c r="P17" s="9">
+      <c r="O17" s="9"/>
+      <c r="P17">
         <v>0.3</v>
       </c>
-      <c r="Q17" s="15">
+      <c r="Q17" s="11">
         <v>0.3</v>
       </c>
-      <c r="R17" s="15">
+      <c r="R17" s="11">
         <v>0.3</v>
       </c>
-      <c r="S17" s="15">
+      <c r="S17" s="11">
         <v>0.3</v>
       </c>
-      <c r="T17" s="15">
+      <c r="T17" s="11">
         <v>0.3</v>
       </c>
-      <c r="U17" s="15">
+      <c r="U17" s="11">
         <v>0.3</v>
       </c>
-      <c r="V17" s="15">
+      <c r="V17" s="11">
         <v>0.3</v>
       </c>
-      <c r="W17" s="15">
+      <c r="W17" s="11">
         <v>0.3</v>
       </c>
-      <c r="X17" s="15">
+      <c r="X17" s="11">
         <v>0.3</v>
       </c>
-      <c r="Y17" s="15">
+      <c r="Y17" s="11">
         <v>0.3</v>
       </c>
-      <c r="Z17" s="15">
+      <c r="Z17" s="11">
         <v>0.3</v>
       </c>
-      <c r="AA17" s="15">
+      <c r="AA17" s="11">
         <v>0.3</v>
       </c>
-      <c r="AB17" s="15">
+      <c r="AB17" s="11">
         <v>0.3</v>
       </c>
-      <c r="AC17" s="15">
+      <c r="AC17" s="11">
         <v>0.3</v>
       </c>
-      <c r="AD17" s="15">
+      <c r="AD17" s="11">
         <v>0.3</v>
       </c>
     </row>
@@ -2529,86 +2524,86 @@
       <c r="C18" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="6">
         <f>1000*D15*D7</f>
         <v>674522520</v>
       </c>
-      <c r="E18" s="10">
-        <v>0</v>
-      </c>
-      <c r="F18" s="10">
-        <v>0</v>
-      </c>
-      <c r="G18" s="10">
-        <v>0</v>
-      </c>
-      <c r="H18" s="10">
-        <v>0</v>
-      </c>
-      <c r="I18" s="10">
-        <v>0</v>
-      </c>
-      <c r="J18" s="10">
-        <v>0</v>
-      </c>
-      <c r="K18" s="10">
-        <v>0</v>
-      </c>
-      <c r="L18" s="10">
-        <v>0</v>
-      </c>
-      <c r="M18" s="10">
-        <v>0</v>
-      </c>
-      <c r="N18" s="10">
-        <v>0</v>
-      </c>
-      <c r="O18" s="10">
+      <c r="E18" s="6">
+        <v>0</v>
+      </c>
+      <c r="F18" s="6">
+        <v>0</v>
+      </c>
+      <c r="G18" s="6">
+        <v>0</v>
+      </c>
+      <c r="H18" s="6">
+        <v>0</v>
+      </c>
+      <c r="I18" s="6">
+        <v>0</v>
+      </c>
+      <c r="J18" s="6">
+        <v>0</v>
+      </c>
+      <c r="K18" s="6">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6">
+        <v>0</v>
+      </c>
+      <c r="M18" s="6">
+        <v>0</v>
+      </c>
+      <c r="N18" s="6">
+        <v>0</v>
+      </c>
+      <c r="O18" s="6">
         <v>-1</v>
       </c>
-      <c r="P18" s="10">
+      <c r="P18" s="6">
         <v>-1</v>
       </c>
-      <c r="Q18" s="10">
+      <c r="Q18" s="6">
         <v>-1</v>
       </c>
-      <c r="R18" s="10">
+      <c r="R18" s="6">
         <v>-1</v>
       </c>
-      <c r="S18" s="10">
+      <c r="S18" s="6">
         <v>-1</v>
       </c>
-      <c r="T18" s="10">
+      <c r="T18" s="6">
         <v>-1</v>
       </c>
-      <c r="U18" s="10">
+      <c r="U18" s="6">
         <v>-1</v>
       </c>
-      <c r="V18" s="10">
+      <c r="V18" s="6">
         <v>-1</v>
       </c>
-      <c r="W18" s="10">
+      <c r="W18" s="6">
         <v>-1</v>
       </c>
-      <c r="X18" s="10">
+      <c r="X18" s="6">
         <v>-1</v>
       </c>
-      <c r="Y18" s="10">
+      <c r="Y18" s="6">
         <v>-1</v>
       </c>
-      <c r="Z18" s="10">
+      <c r="Z18" s="6">
         <v>-1</v>
       </c>
-      <c r="AA18" s="10">
+      <c r="AA18" s="6">
         <v>-1</v>
       </c>
-      <c r="AB18" s="10">
+      <c r="AB18" s="6">
         <v>-1</v>
       </c>
-      <c r="AC18" s="10">
+      <c r="AC18" s="6">
         <v>-1</v>
       </c>
-      <c r="AD18" s="10">
+      <c r="AD18" s="6">
         <v>-1</v>
       </c>
     </row>
@@ -2625,91 +2620,91 @@
       <c r="D19">
         <v>1</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="4">
         <v>0.97</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19">
         <v>0.97</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19">
         <v>0.97</v>
       </c>
-      <c r="H19" s="4">
+      <c r="H19">
         <v>0.97</v>
       </c>
-      <c r="I19" s="4">
+      <c r="I19">
         <v>0.97</v>
       </c>
-      <c r="J19" s="4">
+      <c r="J19">
         <v>0.97</v>
       </c>
-      <c r="K19" s="4">
+      <c r="K19">
         <v>0.97</v>
       </c>
-      <c r="L19" s="4">
+      <c r="L19">
         <v>0.97</v>
       </c>
-      <c r="M19" s="4">
+      <c r="M19">
         <v>0.97</v>
       </c>
-      <c r="N19" s="4">
+      <c r="N19">
         <v>0.97</v>
       </c>
-      <c r="O19" s="4">
+      <c r="O19">
         <v>0.96</v>
       </c>
-      <c r="P19" s="4">
+      <c r="P19">
         <v>0.96</v>
       </c>
-      <c r="Q19" s="15">
+      <c r="Q19" s="11">
         <v>0.96</v>
       </c>
-      <c r="R19" s="15">
+      <c r="R19" s="11">
         <v>0.96</v>
       </c>
-      <c r="S19" s="15">
+      <c r="S19" s="11">
         <v>0.96</v>
       </c>
-      <c r="T19" s="15">
+      <c r="T19" s="11">
         <v>0.96</v>
       </c>
-      <c r="U19" s="15">
+      <c r="U19" s="11">
         <v>0.96</v>
       </c>
-      <c r="V19" s="15">
+      <c r="V19" s="11">
         <v>0.96</v>
       </c>
-      <c r="W19" s="15">
+      <c r="W19" s="11">
         <v>0.96</v>
       </c>
-      <c r="X19" s="15">
+      <c r="X19" s="11">
         <v>0.96</v>
       </c>
-      <c r="Y19" s="15">
+      <c r="Y19" s="11">
         <v>0.96</v>
       </c>
-      <c r="Z19" s="15">
+      <c r="Z19" s="11">
         <v>0.96</v>
       </c>
-      <c r="AA19" s="15">
+      <c r="AA19" s="11">
         <v>0.96</v>
       </c>
-      <c r="AB19" s="15">
+      <c r="AB19" s="11">
         <v>0.96</v>
       </c>
-      <c r="AC19" s="15">
+      <c r="AC19" s="11">
         <v>0.96</v>
       </c>
-      <c r="AD19" s="15">
+      <c r="AD19" s="11">
         <v>0.96</v>
       </c>
       <c r="AE19" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:31">
       <c r="A20" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>44</v>
@@ -2717,85 +2712,85 @@
       <c r="C20" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="6">
         <v>1</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="4">
         <v>1</v>
       </c>
-      <c r="F20" s="10">
+      <c r="F20" s="6">
         <v>1</v>
       </c>
-      <c r="G20" s="10">
+      <c r="G20" s="6">
         <v>1</v>
       </c>
-      <c r="H20" s="10">
+      <c r="H20" s="6">
         <v>1</v>
       </c>
-      <c r="I20" s="10">
+      <c r="I20" s="6">
         <v>1</v>
       </c>
-      <c r="J20" s="10">
+      <c r="J20" s="6">
         <v>1</v>
       </c>
-      <c r="K20" s="10">
+      <c r="K20" s="6">
         <v>1</v>
       </c>
-      <c r="L20" s="10">
+      <c r="L20" s="6">
         <v>1</v>
       </c>
-      <c r="M20" s="10">
+      <c r="M20" s="6">
         <v>1</v>
       </c>
-      <c r="N20" s="10">
+      <c r="N20" s="6">
         <v>1</v>
       </c>
-      <c r="O20" s="10">
+      <c r="O20" s="6">
         <v>1</v>
       </c>
-      <c r="P20" s="10">
+      <c r="P20" s="6">
         <v>1</v>
       </c>
-      <c r="Q20" s="15">
+      <c r="Q20" s="11">
         <v>1</v>
       </c>
-      <c r="R20" s="15">
+      <c r="R20" s="11">
         <v>1</v>
       </c>
-      <c r="S20" s="15">
+      <c r="S20" s="11">
         <v>1</v>
       </c>
-      <c r="T20" s="15">
+      <c r="T20" s="11">
         <v>1</v>
       </c>
-      <c r="U20" s="15">
+      <c r="U20" s="11">
         <v>1</v>
       </c>
-      <c r="V20" s="15">
+      <c r="V20" s="11">
         <v>0.99</v>
       </c>
-      <c r="W20" s="15">
+      <c r="W20" s="11">
         <v>0.99</v>
       </c>
-      <c r="X20" s="15">
+      <c r="X20" s="11">
         <v>0.99</v>
       </c>
-      <c r="Y20" s="15">
+      <c r="Y20" s="11">
         <v>0.99</v>
       </c>
-      <c r="Z20" s="15">
+      <c r="Z20" s="11">
         <v>0.99</v>
       </c>
-      <c r="AA20" s="15">
+      <c r="AA20" s="11">
         <v>0.99</v>
       </c>
-      <c r="AB20" s="15">
+      <c r="AB20" s="11">
         <v>0.99</v>
       </c>
-      <c r="AC20" s="15">
+      <c r="AC20" s="11">
         <v>0.99</v>
       </c>
-      <c r="AD20" s="15">
+      <c r="AD20" s="11">
         <v>0.99</v>
       </c>
     </row>
@@ -2818,7 +2813,7 @@
       <c r="F21" s="1">
         <v>0</v>
       </c>
-      <c r="G21" s="7">
+      <c r="G21" s="4">
         <v>0.108</v>
       </c>
       <c r="H21">
@@ -2891,12 +2886,12 @@
         <v>0.108</v>
       </c>
       <c r="AE21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="22" spans="1:31">
       <c r="A22" t="s">
-        <v>76</v>
+        <v>137</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>44</v>
@@ -2913,7 +2908,7 @@
       <c r="F22">
         <v>0</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="5">
         <v>0</v>
       </c>
       <c r="H22" s="1">
@@ -2943,50 +2938,50 @@
       <c r="P22" s="1">
         <v>0</v>
       </c>
-      <c r="Q22" s="16">
-        <v>0</v>
-      </c>
-      <c r="R22" s="16">
-        <v>0</v>
-      </c>
-      <c r="S22" s="16">
-        <v>0</v>
-      </c>
-      <c r="T22" s="16">
-        <v>0</v>
-      </c>
-      <c r="U22" s="16">
-        <v>0</v>
-      </c>
-      <c r="V22" s="16">
-        <v>0</v>
-      </c>
-      <c r="W22" s="16">
-        <v>0</v>
-      </c>
-      <c r="X22" s="16">
-        <v>0</v>
-      </c>
-      <c r="Y22" s="16">
-        <v>0</v>
-      </c>
-      <c r="Z22" s="16">
-        <v>0</v>
-      </c>
-      <c r="AA22" s="16">
-        <v>0</v>
-      </c>
-      <c r="AB22" s="16">
-        <v>0</v>
-      </c>
-      <c r="AC22" s="16">
-        <v>0</v>
-      </c>
-      <c r="AD22" s="16">
+      <c r="Q22" s="12">
+        <v>0</v>
+      </c>
+      <c r="R22" s="12">
+        <v>0</v>
+      </c>
+      <c r="S22" s="12">
+        <v>0</v>
+      </c>
+      <c r="T22" s="12">
+        <v>0</v>
+      </c>
+      <c r="U22" s="12">
+        <v>0</v>
+      </c>
+      <c r="V22" s="12">
+        <v>0</v>
+      </c>
+      <c r="W22" s="12">
+        <v>0</v>
+      </c>
+      <c r="X22" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="12">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="12">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="12">
+        <v>0</v>
+      </c>
+      <c r="AB22" s="12">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="12">
         <v>0</v>
       </c>
       <c r="AE22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:31">
@@ -3038,50 +3033,50 @@
       <c r="P23">
         <v>900</v>
       </c>
-      <c r="Q23" s="15">
+      <c r="Q23" s="11">
         <v>830</v>
       </c>
-      <c r="R23" s="15">
+      <c r="R23" s="11">
         <v>830</v>
       </c>
-      <c r="S23" s="15">
+      <c r="S23" s="11">
         <v>830</v>
       </c>
-      <c r="T23" s="15">
+      <c r="T23" s="11">
         <v>830</v>
       </c>
-      <c r="U23" s="15">
+      <c r="U23" s="11">
         <v>830</v>
       </c>
-      <c r="V23" s="15">
+      <c r="V23" s="11">
         <v>830</v>
       </c>
-      <c r="W23" s="15">
+      <c r="W23" s="11">
         <v>830</v>
       </c>
-      <c r="X23" s="15">
+      <c r="X23" s="11">
         <v>830</v>
       </c>
-      <c r="Y23" s="15">
+      <c r="Y23" s="11">
         <v>830</v>
       </c>
-      <c r="Z23" s="15">
+      <c r="Z23" s="11">
         <v>830</v>
       </c>
-      <c r="AA23" s="15">
+      <c r="AA23" s="11">
         <v>830</v>
       </c>
-      <c r="AB23" s="15">
+      <c r="AB23" s="11">
         <v>830</v>
       </c>
-      <c r="AC23" s="15">
+      <c r="AC23" s="11">
         <v>830</v>
       </c>
-      <c r="AD23" s="15">
+      <c r="AD23" s="11">
         <v>830</v>
       </c>
       <c r="AE23" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:31">
@@ -3133,50 +3128,50 @@
       <c r="P24">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="Q24" s="7">
+      <c r="Q24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="R24" s="7">
+      <c r="R24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="S24" s="7">
+      <c r="S24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="T24" s="7">
+      <c r="T24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="U24" s="7">
+      <c r="U24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="V24" s="7">
+      <c r="V24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="W24" s="7">
+      <c r="W24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="X24" s="7">
+      <c r="X24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="Y24" s="7">
+      <c r="Y24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="Z24" s="7">
+      <c r="Z24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="AA24" s="7">
+      <c r="AA24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="AB24" s="7">
+      <c r="AB24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="AC24" s="7">
+      <c r="AC24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="AD24" s="7">
+      <c r="AD24" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AE24" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25" spans="1:31">
@@ -3213,13 +3208,13 @@
       <c r="K25">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="L25" s="7">
+      <c r="L25" s="4">
         <v>1.6E-2</v>
       </c>
-      <c r="M25" s="9">
+      <c r="M25">
         <v>1.6E-2</v>
       </c>
-      <c r="N25" s="9">
+      <c r="N25">
         <v>1.6E-2</v>
       </c>
       <c r="O25">
@@ -3228,50 +3223,50 @@
       <c r="P25">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="Q25" s="7">
+      <c r="Q25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="R25" s="7">
+      <c r="R25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="S25" s="7">
+      <c r="S25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="T25" s="7">
+      <c r="T25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="U25" s="7">
+      <c r="U25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="V25" s="7">
+      <c r="V25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="W25" s="7">
+      <c r="W25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="X25" s="7">
+      <c r="X25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="Y25" s="7">
+      <c r="Y25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="Z25" s="7">
+      <c r="Z25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="AA25" s="7">
+      <c r="AA25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="AB25" s="7">
+      <c r="AB25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="AC25" s="7">
+      <c r="AC25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="AD25" s="7">
+      <c r="AD25" s="4">
         <v>2.5999999999999999E-3</v>
       </c>
       <c r="AE25" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="26" spans="1:31">
@@ -3308,13 +3303,13 @@
       <c r="K26">
         <v>0.05</v>
       </c>
-      <c r="L26" s="7">
+      <c r="L26" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="M26" s="7">
+      <c r="M26" s="4">
         <v>1.15E-2</v>
       </c>
-      <c r="N26" s="12">
+      <c r="N26" s="8">
         <v>1.15E-2</v>
       </c>
       <c r="O26">
@@ -3323,50 +3318,50 @@
       <c r="P26">
         <v>0.05</v>
       </c>
-      <c r="Q26" s="7">
+      <c r="Q26" s="4">
         <v>0.05</v>
       </c>
-      <c r="R26" s="7">
+      <c r="R26" s="4">
         <v>0.05</v>
       </c>
-      <c r="S26" s="7">
+      <c r="S26" s="4">
         <v>0.05</v>
       </c>
-      <c r="T26" s="7">
+      <c r="T26" s="4">
         <v>0.05</v>
       </c>
-      <c r="U26" s="7">
+      <c r="U26" s="4">
         <v>0.05</v>
       </c>
-      <c r="V26" s="7">
+      <c r="V26" s="4">
         <v>0.05</v>
       </c>
-      <c r="W26" s="7">
+      <c r="W26" s="4">
         <v>0.05</v>
       </c>
-      <c r="X26" s="7">
+      <c r="X26" s="4">
         <v>0.05</v>
       </c>
-      <c r="Y26" s="7">
+      <c r="Y26" s="4">
         <v>0.05</v>
       </c>
-      <c r="Z26" s="7">
+      <c r="Z26" s="4">
         <v>0.05</v>
       </c>
-      <c r="AA26" s="7">
+      <c r="AA26" s="4">
         <v>0.05</v>
       </c>
-      <c r="AB26" s="7">
+      <c r="AB26" s="4">
         <v>0.05</v>
       </c>
-      <c r="AC26" s="7">
+      <c r="AC26" s="4">
         <v>0.05</v>
       </c>
-      <c r="AD26" s="7">
+      <c r="AD26" s="4">
         <v>0.05</v>
       </c>
       <c r="AE26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="27" spans="1:31">
@@ -3418,50 +3413,50 @@
       <c r="P27">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="Q27" s="7">
+      <c r="Q27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="R27" s="7">
+      <c r="R27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="S27" s="7">
+      <c r="S27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="T27" s="7">
+      <c r="T27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="U27" s="7">
+      <c r="U27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="V27" s="7">
+      <c r="V27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="W27" s="7">
+      <c r="W27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="X27" s="7">
+      <c r="X27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="Y27" s="7">
+      <c r="Y27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="Z27" s="7">
+      <c r="Z27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="AA27" s="7">
+      <c r="AA27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="AB27" s="7">
+      <c r="AB27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="AC27" s="7">
+      <c r="AC27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="AD27" s="7">
+      <c r="AD27" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
       <c r="AE27" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="28" spans="1:31">
@@ -3513,50 +3508,50 @@
       <c r="P28">
         <v>1.9E-2</v>
       </c>
-      <c r="Q28" s="7">
+      <c r="Q28" s="4">
         <v>1.9E-2</v>
       </c>
-      <c r="R28" s="7">
+      <c r="R28" s="4">
         <v>1.9E-2</v>
       </c>
-      <c r="S28" s="7">
+      <c r="S28" s="4">
         <v>1.9E-2</v>
       </c>
-      <c r="T28" s="7">
+      <c r="T28" s="4">
         <v>1.9E-2</v>
       </c>
-      <c r="U28" s="7">
+      <c r="U28" s="4">
         <v>1.9E-2</v>
       </c>
-      <c r="V28" s="7">
+      <c r="V28" s="4">
         <v>1.9E-2</v>
       </c>
-      <c r="W28" s="7">
+      <c r="W28" s="4">
         <v>1.9E-2</v>
       </c>
-      <c r="X28" s="7">
+      <c r="X28" s="4">
         <v>1.9E-2</v>
       </c>
-      <c r="Y28" s="7">
+      <c r="Y28" s="4">
         <v>1.9E-2</v>
       </c>
-      <c r="Z28" s="7">
+      <c r="Z28" s="4">
         <v>1.9E-2</v>
       </c>
-      <c r="AA28" s="7">
+      <c r="AA28" s="4">
         <v>1.9E-2</v>
       </c>
-      <c r="AB28" s="7">
+      <c r="AB28" s="4">
         <v>1.9E-2</v>
       </c>
-      <c r="AC28" s="7">
+      <c r="AC28" s="4">
         <v>1.9E-2</v>
       </c>
-      <c r="AD28" s="7">
+      <c r="AD28" s="4">
         <v>1.9E-2</v>
       </c>
       <c r="AE28" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="29" spans="1:31">
@@ -3572,162 +3567,153 @@
       <c r="D29">
         <v>1100</v>
       </c>
-      <c r="E29" s="4">
+      <c r="E29">
         <v>1100</v>
       </c>
-      <c r="F29" s="4">
+      <c r="F29">
         <v>1100</v>
       </c>
-      <c r="G29" s="4">
+      <c r="G29">
         <v>1100</v>
       </c>
-      <c r="H29" s="5">
+      <c r="H29" s="4">
         <v>3688</v>
       </c>
-      <c r="I29" s="6">
+      <c r="I29">
         <v>3688</v>
       </c>
-      <c r="J29" s="5">
+      <c r="J29" s="4">
         <v>1100</v>
       </c>
-      <c r="K29" s="5">
+      <c r="K29" s="4">
         <v>3688</v>
       </c>
-      <c r="L29" s="6">
+      <c r="L29">
         <v>3688</v>
       </c>
-      <c r="M29" s="6">
+      <c r="M29">
         <v>3688</v>
       </c>
-      <c r="N29" s="6">
+      <c r="N29">
         <v>3688</v>
       </c>
-      <c r="O29" s="6">
+      <c r="O29">
         <v>3688</v>
       </c>
-      <c r="P29" s="6">
+      <c r="P29">
         <v>3688</v>
       </c>
-      <c r="Q29" s="7">
+      <c r="Q29" s="4">
         <v>4917.333333333333</v>
       </c>
-      <c r="R29" s="7">
+      <c r="R29" s="4">
         <v>2634.2857142857142</v>
       </c>
-      <c r="S29" s="7">
+      <c r="S29" s="4">
         <v>6500</v>
       </c>
-      <c r="T29" s="7">
+      <c r="T29" s="4">
         <v>2634.2857142857142</v>
       </c>
-      <c r="U29" s="7">
+      <c r="U29" s="4">
         <v>4917.333333333333</v>
       </c>
-      <c r="V29" s="7">
+      <c r="V29" s="4">
         <v>6500</v>
       </c>
-      <c r="W29" s="7">
+      <c r="W29" s="4">
         <v>3100</v>
       </c>
-      <c r="X29" s="7">
+      <c r="X29" s="4">
         <v>2634.2857142857142</v>
       </c>
-      <c r="Y29" s="19">
+      <c r="Y29" s="9">
         <v>3688</v>
       </c>
-      <c r="Z29" s="19">
+      <c r="Z29" s="9">
         <v>3688</v>
       </c>
-      <c r="AA29" s="7">
+      <c r="AA29" s="4">
         <v>6500</v>
       </c>
-      <c r="AB29" s="7">
+      <c r="AB29" s="4">
         <v>2634.2857142857142</v>
       </c>
-      <c r="AC29" s="7">
+      <c r="AC29" s="4">
         <v>6500</v>
       </c>
-      <c r="AD29" s="7">
+      <c r="AD29" s="4">
         <v>2634.2857142857142</v>
       </c>
       <c r="AE29" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="30" spans="1:31">
       <c r="A30" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>44</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="6"/>
-      <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
-      <c r="L30" s="6"/>
-      <c r="M30" s="6"/>
-      <c r="N30" s="6"/>
-      <c r="O30" s="6"/>
-      <c r="P30" s="6"/>
-      <c r="Q30" s="18">
+        <v>114</v>
+      </c>
+      <c r="H30" s="4"/>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4"/>
+      <c r="Q30" s="14">
         <v>0.37740000000000001</v>
       </c>
-      <c r="R30" s="18">
+      <c r="R30" s="14">
         <v>0.37740000000000001</v>
       </c>
-      <c r="S30" s="18">
+      <c r="S30" s="14">
         <v>0.37740000000000001</v>
       </c>
-      <c r="T30" s="7">
+      <c r="T30" s="4">
         <v>-1</v>
       </c>
-      <c r="U30" s="7">
+      <c r="U30" s="4">
         <v>0.42699999999999999</v>
       </c>
-      <c r="V30" s="7">
+      <c r="V30" s="4">
         <v>0.42699999999999999</v>
       </c>
-      <c r="W30" s="7">
+      <c r="W30" s="4">
         <v>0.39100000000000001</v>
       </c>
-      <c r="X30" s="7">
+      <c r="X30" s="4">
         <v>0.39100000000000001</v>
       </c>
-      <c r="Y30" s="7">
+      <c r="Y30" s="4">
         <v>0.38400000000000001</v>
       </c>
-      <c r="Z30" s="7">
+      <c r="Z30" s="4">
         <v>0.38400000000000001</v>
       </c>
-      <c r="AA30" s="7">
+      <c r="AA30" s="4">
         <v>0.42699999999999999</v>
       </c>
-      <c r="AB30" s="7">
+      <c r="AB30" s="4">
         <v>0.39100000000000001</v>
       </c>
-      <c r="AC30" s="7">
+      <c r="AC30" s="4">
         <v>0.42699999999999999</v>
       </c>
-      <c r="AD30" s="7">
+      <c r="AD30" s="4">
         <v>0.39100000000000001</v>
       </c>
     </row>
     <row r="31" spans="1:31">
       <c r="A31" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>44</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D31">
         <v>0.98</v>
@@ -3824,86 +3810,86 @@
       <c r="D32">
         <v>385</v>
       </c>
-      <c r="E32" s="4">
+      <c r="E32">
         <v>385</v>
       </c>
-      <c r="F32" s="4">
+      <c r="F32">
         <v>385</v>
       </c>
-      <c r="G32" s="4">
+      <c r="G32">
         <v>385</v>
       </c>
-      <c r="H32" s="6">
+      <c r="H32">
         <v>385</v>
       </c>
-      <c r="I32" s="6">
+      <c r="I32">
         <v>385</v>
       </c>
-      <c r="J32" s="6">
+      <c r="J32">
         <v>385</v>
       </c>
-      <c r="K32" s="6">
+      <c r="K32">
         <v>385</v>
       </c>
-      <c r="L32" s="6">
+      <c r="L32">
         <v>385</v>
       </c>
-      <c r="M32" s="6">
+      <c r="M32">
         <v>385</v>
       </c>
-      <c r="N32" s="6">
+      <c r="N32">
         <v>385</v>
       </c>
-      <c r="O32" s="6">
+      <c r="O32">
         <v>550</v>
       </c>
-      <c r="P32" s="6">
+      <c r="P32">
         <v>550</v>
       </c>
-      <c r="Q32" s="7">
+      <c r="Q32" s="4">
         <v>560</v>
       </c>
-      <c r="R32" s="15">
+      <c r="R32" s="11">
         <v>405</v>
       </c>
-      <c r="S32" s="7">
+      <c r="S32" s="4">
         <v>560</v>
       </c>
-      <c r="T32" s="15">
+      <c r="T32" s="11">
         <v>405</v>
       </c>
-      <c r="U32" s="7">
+      <c r="U32" s="4">
         <v>560</v>
       </c>
-      <c r="V32" s="7">
+      <c r="V32" s="4">
         <v>560</v>
       </c>
-      <c r="W32" s="15">
+      <c r="W32" s="11">
         <v>405</v>
       </c>
-      <c r="X32" s="15">
+      <c r="X32" s="11">
         <v>405</v>
       </c>
-      <c r="Y32" s="7">
+      <c r="Y32" s="4">
         <v>385</v>
       </c>
-      <c r="Z32" s="7">
+      <c r="Z32" s="4">
         <v>385</v>
       </c>
-      <c r="AA32" s="7">
+      <c r="AA32" s="4">
         <v>560</v>
       </c>
-      <c r="AB32" s="15">
+      <c r="AB32" s="11">
         <v>405</v>
       </c>
-      <c r="AC32" s="7">
+      <c r="AC32" s="4">
         <v>560</v>
       </c>
-      <c r="AD32" s="15">
+      <c r="AD32" s="11">
         <v>405</v>
       </c>
       <c r="AE32" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="33" spans="1:31">
@@ -3919,86 +3905,86 @@
       <c r="D33">
         <v>15</v>
       </c>
-      <c r="E33" s="5">
+      <c r="E33" s="4">
         <v>60</v>
       </c>
-      <c r="F33" s="4">
+      <c r="F33">
         <v>60</v>
       </c>
-      <c r="G33" s="4">
+      <c r="G33">
         <v>60</v>
       </c>
-      <c r="H33" s="4">
+      <c r="H33">
         <v>60</v>
       </c>
-      <c r="I33" s="4">
+      <c r="I33">
         <v>60</v>
       </c>
-      <c r="J33" s="4">
+      <c r="J33">
         <v>60</v>
       </c>
-      <c r="K33" s="4">
+      <c r="K33">
         <v>60</v>
       </c>
-      <c r="L33" s="4">
+      <c r="L33">
         <v>60</v>
       </c>
-      <c r="M33" s="4">
+      <c r="M33">
         <v>60</v>
       </c>
-      <c r="N33" s="4">
+      <c r="N33">
         <v>60</v>
       </c>
-      <c r="O33" s="4">
+      <c r="O33">
         <v>260</v>
       </c>
-      <c r="P33" s="4">
+      <c r="P33">
         <v>260</v>
       </c>
-      <c r="Q33" s="7">
+      <c r="Q33" s="4">
         <v>260</v>
       </c>
-      <c r="R33" s="15">
+      <c r="R33" s="11">
         <v>-20</v>
       </c>
-      <c r="S33" s="7">
+      <c r="S33" s="4">
         <v>260</v>
       </c>
-      <c r="T33" s="15">
+      <c r="T33" s="11">
         <v>-20</v>
       </c>
-      <c r="U33" s="7">
+      <c r="U33" s="4">
         <v>260</v>
       </c>
-      <c r="V33" s="7">
+      <c r="V33" s="4">
         <v>260</v>
       </c>
-      <c r="W33" s="15">
+      <c r="W33" s="11">
         <v>-20</v>
       </c>
-      <c r="X33" s="15">
+      <c r="X33" s="11">
         <v>-20</v>
       </c>
-      <c r="Y33" s="7">
+      <c r="Y33" s="4">
         <v>60</v>
       </c>
-      <c r="Z33" s="7">
+      <c r="Z33" s="4">
         <v>60</v>
       </c>
-      <c r="AA33" s="7">
+      <c r="AA33" s="4">
         <v>260</v>
       </c>
-      <c r="AB33" s="15">
+      <c r="AB33" s="11">
         <v>-20</v>
       </c>
-      <c r="AC33" s="7">
+      <c r="AC33" s="4">
         <v>260</v>
       </c>
-      <c r="AD33" s="15">
+      <c r="AD33" s="11">
         <v>-20</v>
       </c>
       <c r="AE33" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="34" spans="1:31">
@@ -4044,67 +4030,67 @@
       <c r="N34">
         <v>295</v>
       </c>
-      <c r="O34" s="4">
+      <c r="O34">
         <v>295</v>
       </c>
-      <c r="P34" s="4">
+      <c r="P34">
         <v>295</v>
       </c>
-      <c r="Q34" s="7">
+      <c r="Q34" s="4">
         <v>290</v>
       </c>
-      <c r="R34" s="15">
+      <c r="R34" s="11">
         <v>290</v>
       </c>
-      <c r="S34" s="7">
+      <c r="S34" s="4">
         <v>290</v>
       </c>
-      <c r="T34" s="15">
+      <c r="T34" s="11">
         <v>290</v>
       </c>
-      <c r="U34" s="7">
+      <c r="U34" s="4">
         <v>290</v>
       </c>
-      <c r="V34" s="7">
+      <c r="V34" s="4">
         <v>290</v>
       </c>
-      <c r="W34" s="15">
+      <c r="W34" s="11">
         <v>290</v>
       </c>
-      <c r="X34" s="15">
+      <c r="X34" s="11">
         <v>290</v>
       </c>
-      <c r="Y34" s="7">
+      <c r="Y34" s="4">
         <v>290</v>
       </c>
-      <c r="Z34" s="7">
+      <c r="Z34" s="4">
         <v>290</v>
       </c>
-      <c r="AA34" s="7">
+      <c r="AA34" s="4">
         <v>290</v>
       </c>
-      <c r="AB34" s="15">
+      <c r="AB34" s="11">
         <v>290</v>
       </c>
-      <c r="AC34" s="7">
+      <c r="AC34" s="4">
         <v>290</v>
       </c>
-      <c r="AD34" s="15">
+      <c r="AD34" s="11">
         <v>290</v>
       </c>
       <c r="AE34" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="35" spans="1:31">
       <c r="A35" t="s">
+        <v>76</v>
+      </c>
+      <c r="B35" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="C35" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>79</v>
       </c>
       <c r="D35">
         <v>40</v>
@@ -4190,737 +4176,737 @@
     </row>
     <row r="36" spans="1:31">
       <c r="A36" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D36" s="17">
+        <v>102</v>
+      </c>
+      <c r="D36" s="13">
         <v>1140</v>
       </c>
-      <c r="E36" s="17">
+      <c r="E36" s="13">
         <v>1140</v>
       </c>
-      <c r="F36" s="17">
+      <c r="F36" s="13">
         <v>1140</v>
       </c>
-      <c r="G36" s="17">
+      <c r="G36" s="13">
         <v>1140</v>
       </c>
-      <c r="H36" s="17">
+      <c r="H36" s="13">
         <v>1140</v>
       </c>
-      <c r="I36" s="17">
+      <c r="I36" s="13">
         <v>1140</v>
       </c>
-      <c r="J36" s="17">
+      <c r="J36" s="13">
         <v>1140</v>
       </c>
-      <c r="K36" s="17">
+      <c r="K36" s="13">
         <v>1140</v>
       </c>
-      <c r="L36" s="17">
+      <c r="L36" s="13">
         <v>1140</v>
       </c>
-      <c r="M36" s="17">
+      <c r="M36" s="13">
         <v>1140</v>
       </c>
-      <c r="N36" s="17">
+      <c r="N36" s="13">
         <v>1140</v>
       </c>
-      <c r="O36" s="17">
+      <c r="O36" s="13">
         <v>1140</v>
       </c>
-      <c r="P36" s="17">
+      <c r="P36" s="13">
         <v>1140</v>
       </c>
-      <c r="Q36" s="15">
+      <c r="Q36" s="11">
         <v>1140</v>
       </c>
-      <c r="R36" s="15">
+      <c r="R36" s="11">
         <v>1140</v>
       </c>
-      <c r="S36" s="15">
+      <c r="S36" s="11">
         <v>1140</v>
       </c>
-      <c r="T36" s="15">
+      <c r="T36" s="11">
         <v>1140</v>
       </c>
-      <c r="U36" s="15">
+      <c r="U36" s="11">
         <v>1220</v>
       </c>
-      <c r="V36" s="15">
+      <c r="V36" s="11">
         <v>1003.2</v>
       </c>
-      <c r="W36" s="15">
+      <c r="W36" s="11">
         <v>1003.2</v>
       </c>
-      <c r="X36" s="15">
+      <c r="X36" s="11">
         <v>1003.2</v>
       </c>
-      <c r="Y36" s="15">
+      <c r="Y36" s="11">
         <v>1056</v>
       </c>
-      <c r="Z36" s="15">
+      <c r="Z36" s="11">
         <v>1003.2</v>
       </c>
-      <c r="AA36" s="15">
+      <c r="AA36" s="11">
         <v>922.94399999999996</v>
       </c>
-      <c r="AB36" s="15">
+      <c r="AB36" s="11">
         <v>922.94399999999996</v>
       </c>
-      <c r="AC36" s="15">
+      <c r="AC36" s="11">
         <v>882.81600000000003</v>
       </c>
-      <c r="AD36" s="15">
+      <c r="AD36" s="11">
         <v>882.81600000000003</v>
       </c>
     </row>
     <row r="37" spans="1:31">
       <c r="A37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D37" s="17">
+        <v>102</v>
+      </c>
+      <c r="D37" s="13">
         <v>29</v>
       </c>
-      <c r="E37" s="17">
+      <c r="E37" s="13">
         <v>29</v>
       </c>
-      <c r="F37" s="17">
+      <c r="F37" s="13">
         <v>29</v>
       </c>
-      <c r="G37" s="17">
+      <c r="G37" s="13">
         <v>29</v>
       </c>
-      <c r="H37" s="17">
+      <c r="H37" s="13">
         <v>29</v>
       </c>
-      <c r="I37" s="17">
+      <c r="I37" s="13">
         <v>29</v>
       </c>
-      <c r="J37" s="17">
+      <c r="J37" s="13">
         <v>29</v>
       </c>
-      <c r="K37" s="17">
+      <c r="K37" s="13">
         <v>29</v>
       </c>
-      <c r="L37" s="17">
+      <c r="L37" s="13">
         <v>29</v>
       </c>
-      <c r="M37" s="17">
+      <c r="M37" s="13">
         <v>29</v>
       </c>
-      <c r="N37" s="17">
+      <c r="N37" s="13">
         <v>29</v>
       </c>
-      <c r="O37" s="17">
+      <c r="O37" s="13">
         <v>29</v>
       </c>
-      <c r="P37" s="17">
+      <c r="P37" s="13">
         <v>29</v>
       </c>
-      <c r="Q37" s="7">
+      <c r="Q37" s="4">
         <v>29</v>
       </c>
-      <c r="R37" s="15">
+      <c r="R37" s="11">
         <v>42</v>
       </c>
-      <c r="S37" s="7">
+      <c r="S37" s="4">
         <v>29</v>
       </c>
-      <c r="T37" s="15">
+      <c r="T37" s="11">
         <v>42</v>
       </c>
-      <c r="U37" s="7">
+      <c r="U37" s="4">
         <v>42</v>
       </c>
-      <c r="V37" s="7">
+      <c r="V37" s="4">
         <v>25.52</v>
       </c>
-      <c r="W37" s="15">
+      <c r="W37" s="11">
         <v>36.96</v>
       </c>
-      <c r="X37" s="15">
+      <c r="X37" s="11">
         <v>36.96</v>
       </c>
-      <c r="Y37" s="7">
+      <c r="Y37" s="4">
         <v>44</v>
       </c>
-      <c r="Z37" s="7">
+      <c r="Z37" s="4">
         <v>36.96</v>
       </c>
-      <c r="AA37" s="7">
+      <c r="AA37" s="4">
         <v>23.478400000000001</v>
       </c>
-      <c r="AB37" s="15">
+      <c r="AB37" s="11">
         <v>34.0032</v>
       </c>
-      <c r="AC37" s="7">
+      <c r="AC37" s="4">
         <v>22.457599999999999</v>
       </c>
-      <c r="AD37" s="15">
+      <c r="AD37" s="11">
         <v>32.524799999999999</v>
       </c>
     </row>
     <row r="38" spans="1:31">
       <c r="A38" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D38" s="17">
+        <v>102</v>
+      </c>
+      <c r="D38" s="13">
         <v>188</v>
       </c>
-      <c r="E38" s="17">
+      <c r="E38" s="13">
         <v>188</v>
       </c>
-      <c r="F38" s="17">
+      <c r="F38" s="13">
         <v>188</v>
       </c>
-      <c r="G38" s="17">
+      <c r="G38" s="13">
         <v>188</v>
       </c>
-      <c r="H38" s="17">
+      <c r="H38" s="13">
         <v>188</v>
       </c>
-      <c r="I38" s="17">
+      <c r="I38" s="13">
         <v>188</v>
       </c>
-      <c r="J38" s="17">
+      <c r="J38" s="13">
         <v>188</v>
       </c>
-      <c r="K38" s="17">
+      <c r="K38" s="13">
         <v>188</v>
       </c>
-      <c r="L38" s="17">
+      <c r="L38" s="13">
         <v>188</v>
       </c>
-      <c r="M38" s="17">
+      <c r="M38" s="13">
         <v>188</v>
       </c>
-      <c r="N38" s="17">
+      <c r="N38" s="13">
         <v>188</v>
       </c>
-      <c r="O38" s="17">
+      <c r="O38" s="13">
         <v>188</v>
       </c>
-      <c r="P38" s="17">
+      <c r="P38" s="13">
         <v>188</v>
       </c>
-      <c r="Q38" s="7">
+      <c r="Q38" s="4">
         <v>188</v>
       </c>
-      <c r="R38" s="15">
+      <c r="R38" s="11">
         <v>219</v>
       </c>
-      <c r="S38" s="7">
+      <c r="S38" s="4">
         <v>188</v>
       </c>
-      <c r="T38" s="15">
+      <c r="T38" s="11">
         <v>219</v>
       </c>
-      <c r="U38" s="7">
+      <c r="U38" s="4">
         <v>231</v>
       </c>
-      <c r="V38" s="7">
+      <c r="V38" s="4">
         <v>165.44</v>
       </c>
-      <c r="W38" s="15">
+      <c r="W38" s="11">
         <v>192.72</v>
       </c>
-      <c r="X38" s="15">
+      <c r="X38" s="11">
         <v>192.72</v>
       </c>
-      <c r="Y38" s="7">
+      <c r="Y38" s="4">
         <v>220</v>
       </c>
-      <c r="Z38" s="7">
+      <c r="Z38" s="4">
         <v>172.21600000000001</v>
       </c>
-      <c r="AA38" s="7">
+      <c r="AA38" s="4">
         <v>152.19999999999999</v>
       </c>
-      <c r="AB38" s="15">
+      <c r="AB38" s="11">
         <v>177.30240000000001</v>
       </c>
-      <c r="AC38" s="7">
+      <c r="AC38" s="4">
         <v>145.5872</v>
       </c>
-      <c r="AD38" s="15">
+      <c r="AD38" s="11">
         <v>169.59360000000001</v>
       </c>
     </row>
     <row r="39" spans="1:31">
       <c r="A39" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D39" s="17">
+        <v>102</v>
+      </c>
+      <c r="D39" s="13">
         <v>1</v>
       </c>
-      <c r="E39" s="17">
+      <c r="E39" s="13">
         <v>1</v>
       </c>
-      <c r="F39" s="17">
+      <c r="F39" s="13">
         <v>1</v>
       </c>
-      <c r="G39" s="17">
+      <c r="G39" s="13">
         <v>1</v>
       </c>
-      <c r="H39" s="17">
+      <c r="H39" s="13">
         <v>1</v>
       </c>
-      <c r="I39" s="17">
+      <c r="I39" s="13">
         <v>1</v>
       </c>
-      <c r="J39" s="17">
+      <c r="J39" s="13">
         <v>1</v>
       </c>
-      <c r="K39" s="17">
+      <c r="K39" s="13">
         <v>1</v>
       </c>
-      <c r="L39" s="17">
+      <c r="L39" s="13">
         <v>1</v>
       </c>
-      <c r="M39" s="17">
+      <c r="M39" s="13">
         <v>1</v>
       </c>
-      <c r="N39" s="17">
+      <c r="N39" s="13">
         <v>1</v>
       </c>
-      <c r="O39" s="17">
+      <c r="O39" s="13">
         <v>1</v>
       </c>
-      <c r="P39" s="17">
+      <c r="P39" s="13">
         <v>1</v>
       </c>
-      <c r="Q39" s="7">
+      <c r="Q39" s="4">
         <v>1</v>
       </c>
-      <c r="R39" s="15">
+      <c r="R39" s="11">
         <v>1</v>
       </c>
-      <c r="S39" s="7">
+      <c r="S39" s="4">
         <v>1</v>
       </c>
-      <c r="T39" s="15">
+      <c r="T39" s="11">
         <v>1</v>
       </c>
-      <c r="U39" s="7">
+      <c r="U39" s="4">
         <v>1</v>
       </c>
-      <c r="V39" s="7">
+      <c r="V39" s="4">
         <v>0.88</v>
       </c>
-      <c r="W39" s="15">
+      <c r="W39" s="11">
         <v>0.88</v>
       </c>
-      <c r="X39" s="15">
+      <c r="X39" s="11">
         <v>0.88</v>
       </c>
-      <c r="Y39" s="7">
+      <c r="Y39" s="4">
         <v>0.88</v>
       </c>
-      <c r="Z39" s="7">
+      <c r="Z39" s="4">
         <v>0.88</v>
       </c>
-      <c r="AA39" s="7">
+      <c r="AA39" s="4">
         <v>0.8196</v>
       </c>
-      <c r="AB39" s="15">
+      <c r="AB39" s="11">
         <v>0.8196</v>
       </c>
-      <c r="AC39" s="7">
+      <c r="AC39" s="4">
         <v>0.77439999999999998</v>
       </c>
-      <c r="AD39" s="15">
+      <c r="AD39" s="11">
         <v>0.77439999999999998</v>
       </c>
     </row>
     <row r="40" spans="1:31">
       <c r="A40" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B40" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C40" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D40" s="17">
+      <c r="D40" s="13">
         <v>11</v>
       </c>
-      <c r="E40" s="17">
+      <c r="E40" s="13">
         <v>11</v>
       </c>
-      <c r="F40" s="17">
+      <c r="F40" s="13">
         <v>11</v>
       </c>
-      <c r="G40" s="17">
+      <c r="G40" s="13">
         <v>11</v>
       </c>
-      <c r="H40" s="17">
+      <c r="H40" s="13">
         <v>11</v>
       </c>
-      <c r="I40" s="17">
+      <c r="I40" s="13">
         <v>11</v>
       </c>
-      <c r="J40" s="17">
+      <c r="J40" s="13">
         <v>11</v>
       </c>
-      <c r="K40" s="17">
+      <c r="K40" s="13">
         <v>11</v>
       </c>
-      <c r="L40" s="17">
+      <c r="L40" s="13">
         <v>11</v>
       </c>
-      <c r="M40" s="17">
+      <c r="M40" s="13">
         <v>11</v>
       </c>
-      <c r="N40" s="17">
+      <c r="N40" s="13">
         <v>11</v>
       </c>
-      <c r="O40" s="17">
+      <c r="O40" s="13">
         <v>11</v>
       </c>
-      <c r="P40" s="17">
+      <c r="P40" s="13">
         <v>11</v>
       </c>
-      <c r="Q40" s="7">
+      <c r="Q40" s="4">
         <v>11</v>
       </c>
-      <c r="R40" s="15">
+      <c r="R40" s="11">
         <v>11</v>
       </c>
-      <c r="S40" s="7">
+      <c r="S40" s="4">
         <v>11</v>
       </c>
-      <c r="T40" s="15">
+      <c r="T40" s="11">
         <v>11</v>
       </c>
-      <c r="U40" s="7">
+      <c r="U40" s="4">
         <v>15</v>
       </c>
-      <c r="V40" s="7">
+      <c r="V40" s="4">
         <v>11</v>
       </c>
-      <c r="W40" s="15">
+      <c r="W40" s="11">
         <v>11</v>
       </c>
-      <c r="X40" s="15">
+      <c r="X40" s="11">
         <v>11</v>
       </c>
-      <c r="Y40" s="7">
+      <c r="Y40" s="4">
         <v>15</v>
       </c>
-      <c r="Z40" s="7">
+      <c r="Z40" s="4">
         <v>11</v>
       </c>
-      <c r="AA40" s="7">
+      <c r="AA40" s="4">
         <v>11</v>
       </c>
-      <c r="AB40" s="15">
+      <c r="AB40" s="11">
         <v>11</v>
       </c>
-      <c r="AC40" s="7">
+      <c r="AC40" s="4">
         <v>11</v>
       </c>
-      <c r="AD40" s="15">
+      <c r="AD40" s="11">
         <v>11</v>
       </c>
     </row>
     <row r="41" spans="1:31">
       <c r="A41" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C41" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C41" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D41" s="17">
+      <c r="D41" s="13">
         <v>2</v>
       </c>
-      <c r="E41" s="17">
+      <c r="E41" s="13">
         <v>2</v>
       </c>
-      <c r="F41" s="17">
+      <c r="F41" s="13">
         <v>2</v>
       </c>
-      <c r="G41" s="17">
+      <c r="G41" s="13">
         <v>2</v>
       </c>
-      <c r="H41" s="17">
+      <c r="H41" s="13">
         <v>2</v>
       </c>
-      <c r="I41" s="17">
+      <c r="I41" s="13">
         <v>2</v>
       </c>
-      <c r="J41" s="17">
+      <c r="J41" s="13">
         <v>2</v>
       </c>
-      <c r="K41" s="17">
+      <c r="K41" s="13">
         <v>2</v>
       </c>
-      <c r="L41" s="17">
+      <c r="L41" s="13">
         <v>2</v>
       </c>
-      <c r="M41" s="17">
+      <c r="M41" s="13">
         <v>2</v>
       </c>
-      <c r="N41" s="17">
+      <c r="N41" s="13">
         <v>2</v>
       </c>
-      <c r="O41" s="17">
+      <c r="O41" s="13">
         <v>2</v>
       </c>
-      <c r="P41" s="17">
+      <c r="P41" s="13">
         <v>2</v>
       </c>
-      <c r="Q41" s="7">
+      <c r="Q41" s="4">
         <v>2</v>
       </c>
-      <c r="R41" s="15">
+      <c r="R41" s="11">
         <v>2</v>
       </c>
-      <c r="S41" s="7">
+      <c r="S41" s="4">
         <v>2</v>
       </c>
-      <c r="T41" s="15">
+      <c r="T41" s="11">
         <v>2</v>
       </c>
-      <c r="U41" s="7">
+      <c r="U41" s="4">
         <v>2</v>
       </c>
-      <c r="V41" s="7">
+      <c r="V41" s="4">
         <v>2</v>
       </c>
-      <c r="W41" s="15">
+      <c r="W41" s="11">
         <v>2</v>
       </c>
-      <c r="X41" s="15">
+      <c r="X41" s="11">
         <v>2</v>
       </c>
-      <c r="Y41" s="7">
+      <c r="Y41" s="4">
         <v>2</v>
       </c>
-      <c r="Z41" s="7">
+      <c r="Z41" s="4">
         <v>2</v>
       </c>
-      <c r="AA41" s="7">
+      <c r="AA41" s="4">
         <v>2</v>
       </c>
-      <c r="AB41" s="15">
+      <c r="AB41" s="11">
         <v>2</v>
       </c>
-      <c r="AC41" s="7">
+      <c r="AC41" s="4">
         <v>2</v>
       </c>
-      <c r="AD41" s="15">
+      <c r="AD41" s="11">
         <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:31">
       <c r="A42" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D42" s="17">
+        <v>102</v>
+      </c>
+      <c r="D42" s="13">
         <v>0.04</v>
       </c>
-      <c r="E42" s="17">
+      <c r="E42" s="13">
         <v>0.04</v>
       </c>
-      <c r="F42" s="17">
+      <c r="F42" s="13">
         <v>0.04</v>
       </c>
-      <c r="G42" s="17">
+      <c r="G42" s="13">
         <v>0.04</v>
       </c>
-      <c r="H42" s="17">
+      <c r="H42" s="13">
         <v>0.04</v>
       </c>
-      <c r="I42" s="17">
+      <c r="I42" s="13">
         <v>0.04</v>
       </c>
-      <c r="J42" s="17">
+      <c r="J42" s="13">
         <v>0.04</v>
       </c>
-      <c r="K42" s="17">
+      <c r="K42" s="13">
         <v>0.04</v>
       </c>
-      <c r="L42" s="17">
+      <c r="L42" s="13">
         <v>0.04</v>
       </c>
-      <c r="M42" s="17">
+      <c r="M42" s="13">
         <v>0.04</v>
       </c>
-      <c r="N42" s="17">
+      <c r="N42" s="13">
         <v>0.04</v>
       </c>
-      <c r="O42" s="17">
+      <c r="O42" s="13">
         <v>0.04</v>
       </c>
-      <c r="P42" s="17">
+      <c r="P42" s="13">
         <v>0.04</v>
       </c>
-      <c r="Q42" s="15">
+      <c r="Q42" s="11">
         <v>0.05</v>
       </c>
-      <c r="R42" s="15">
+      <c r="R42" s="11">
         <v>0.05</v>
       </c>
-      <c r="S42" s="15">
+      <c r="S42" s="11">
         <v>0.05</v>
       </c>
-      <c r="T42" s="15">
+      <c r="T42" s="11">
         <v>0.05</v>
       </c>
-      <c r="U42" s="15">
+      <c r="U42" s="11">
         <v>0.05</v>
       </c>
-      <c r="V42" s="15">
+      <c r="V42" s="11">
         <v>0.05</v>
       </c>
-      <c r="W42" s="15">
+      <c r="W42" s="11">
         <v>0.05</v>
       </c>
-      <c r="X42" s="15">
+      <c r="X42" s="11">
         <v>0.05</v>
       </c>
-      <c r="Y42" s="15">
+      <c r="Y42" s="11">
         <v>0.05</v>
       </c>
-      <c r="Z42" s="15">
+      <c r="Z42" s="11">
         <v>0.05</v>
       </c>
-      <c r="AA42" s="15">
+      <c r="AA42" s="11">
         <v>0.05</v>
       </c>
-      <c r="AB42" s="15">
+      <c r="AB42" s="11">
         <v>0.05</v>
       </c>
-      <c r="AC42" s="15">
+      <c r="AC42" s="11">
         <v>0.05</v>
       </c>
-      <c r="AD42" s="15">
+      <c r="AD42" s="11">
         <v>0.05</v>
       </c>
     </row>
     <row r="43" spans="1:31">
       <c r="A43" t="s">
+        <v>103</v>
+      </c>
+      <c r="B43" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="B43" s="3" t="s">
-        <v>105</v>
-      </c>
       <c r="C43" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D43" s="17">
+        <v>102</v>
+      </c>
+      <c r="D43" s="13">
         <v>8</v>
       </c>
-      <c r="E43" s="17">
+      <c r="E43" s="13">
         <v>8</v>
       </c>
-      <c r="F43" s="17">
+      <c r="F43" s="13">
         <v>8</v>
       </c>
-      <c r="G43" s="17">
+      <c r="G43" s="13">
         <v>8</v>
       </c>
-      <c r="H43" s="17">
+      <c r="H43" s="13">
         <v>8</v>
       </c>
-      <c r="I43" s="17">
+      <c r="I43" s="13">
         <v>8</v>
       </c>
-      <c r="J43" s="17">
+      <c r="J43" s="13">
         <v>8</v>
       </c>
-      <c r="K43" s="17">
+      <c r="K43" s="13">
         <v>8</v>
       </c>
-      <c r="L43" s="17">
+      <c r="L43" s="13">
         <v>8</v>
       </c>
-      <c r="M43" s="17">
+      <c r="M43" s="13">
         <v>8</v>
       </c>
-      <c r="N43" s="17">
+      <c r="N43" s="13">
         <v>8</v>
       </c>
-      <c r="O43" s="17">
+      <c r="O43" s="13">
         <v>8</v>
       </c>
-      <c r="P43" s="17">
+      <c r="P43" s="13">
         <v>8</v>
       </c>
-      <c r="Q43" s="15">
+      <c r="Q43" s="11">
         <v>8</v>
       </c>
-      <c r="R43" s="15">
+      <c r="R43" s="11">
         <v>8</v>
       </c>
-      <c r="S43" s="15">
+      <c r="S43" s="11">
         <v>8</v>
       </c>
-      <c r="T43" s="15">
+      <c r="T43" s="11">
         <v>8</v>
       </c>
-      <c r="U43" s="15">
+      <c r="U43" s="11">
         <v>8</v>
       </c>
-      <c r="V43" s="15">
+      <c r="V43" s="11">
         <v>8</v>
       </c>
-      <c r="W43" s="15">
+      <c r="W43" s="11">
         <v>8</v>
       </c>
-      <c r="X43" s="15">
+      <c r="X43" s="11">
         <v>8</v>
       </c>
-      <c r="Y43" s="15">
+      <c r="Y43" s="11">
         <v>8</v>
       </c>
-      <c r="Z43" s="15">
+      <c r="Z43" s="11">
         <v>8</v>
       </c>
-      <c r="AA43" s="15">
+      <c r="AA43" s="11">
         <v>8</v>
       </c>
-      <c r="AB43" s="15">
+      <c r="AB43" s="11">
         <v>8</v>
       </c>
-      <c r="AC43" s="15">
+      <c r="AC43" s="11">
         <v>8</v>
       </c>
-      <c r="AD43" s="15">
+      <c r="AD43" s="11">
         <v>8</v>
       </c>
     </row>
@@ -4949,10 +4935,10 @@
       <c r="H44" t="s">
         <v>60</v>
       </c>
-      <c r="I44" s="7" t="s">
+      <c r="I44" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="J44" s="7" t="s">
+      <c r="J44" s="4" t="s">
         <v>61</v>
       </c>
       <c r="K44" t="s">
@@ -5152,52 +5138,52 @@
         <v>45</v>
       </c>
       <c r="O46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="Q46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="R46" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="S46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="T46" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="U46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="V46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W46" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="X46" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="Y46" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="Z46" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AA46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AB46" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AC46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AD46" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="47" spans="1:31">
@@ -5221,14 +5207,6 @@
       <c r="A48" t="s">
         <v>72</v>
       </c>
-      <c r="I48" s="9"/>
-      <c r="J48" s="9"/>
-      <c r="K48" s="9"/>
-      <c r="L48" s="9"/>
-      <c r="M48" s="9"/>
-      <c r="N48" s="9"/>
-      <c r="O48" s="9"/>
-      <c r="P48" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>